<commit_message>
Observations on the Error Analysis of Diversified and Disturbed dataset Eval
</commit_message>
<xml_diff>
--- a/research/results/121225/summary_eval.xlsx
+++ b/research/results/121225/summary_eval.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Harshit Nigam\Desktop\Coding\Table Diversification\research\results\121225\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33E7FC5-DA36-450C-B6C0-E26757B020C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1724C043-94BD-4DC4-9FDD-956E0424899B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="82">
   <si>
     <t>query_index</t>
   </si>
@@ -264,6 +264,9 @@
   </si>
   <si>
     <t>9/20</t>
+  </si>
+  <si>
+    <t>Success Rate:</t>
   </si>
 </sst>
 </file>
@@ -369,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -378,23 +381,17 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -406,10 +403,15 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1523,13 +1525,13 @@
   <dimension ref="A1:P22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="9.5703125" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" customWidth="1"/>
     <col min="7" max="7" width="9.5703125" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="10.5703125" customWidth="1"/>
-    <col min="10" max="11" width="11.140625" customWidth="1"/>
-    <col min="12" max="12" width="10.85546875" customWidth="1"/>
+    <col min="9" max="10" width="10.5703125" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="10.5703125" customWidth="1"/>
     <col min="15" max="15" width="10.42578125" customWidth="1"/>
     <col min="16" max="16" width="23" customWidth="1"/>
   </cols>
@@ -1600,7 +1602,7 @@
       <c r="I2" t="b">
         <v>1</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="6" t="s">
         <v>62</v>
       </c>
       <c r="K2" t="b">
@@ -1609,10 +1611,10 @@
       <c r="L2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="O2" s="10" t="s">
+      <c r="O2" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="P2" s="10"/>
+      <c r="P2" s="12"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -1651,8 +1653,8 @@
       <c r="L3" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="O3" s="11"/>
-      <c r="P3" s="12" t="s">
+      <c r="O3" s="16"/>
+      <c r="P3" s="11" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1681,7 +1683,7 @@
       <c r="H4" t="b">
         <v>1</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="8" t="s">
         <v>67</v>
       </c>
       <c r="J4" t="b">
@@ -1693,8 +1695,8 @@
       <c r="L4" t="b">
         <v>1</v>
       </c>
-      <c r="O4" s="11"/>
-      <c r="P4" s="12"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="11"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -1730,11 +1732,11 @@
       <c r="K5" t="b">
         <v>1</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="L5" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="O5" s="13"/>
-      <c r="P5" s="12" t="s">
+      <c r="O5" s="17"/>
+      <c r="P5" s="11" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1775,8 +1777,8 @@
       <c r="L6" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="O6" s="13"/>
-      <c r="P6" s="12"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="11"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -1812,11 +1814,11 @@
       <c r="K7" t="b">
         <v>1</v>
       </c>
-      <c r="L7" s="7" t="s">
+      <c r="L7" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="O7" s="14"/>
-      <c r="P7" s="12" t="s">
+      <c r="O7" s="18"/>
+      <c r="P7" s="11" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1836,7 +1838,7 @@
       <c r="E8" t="b">
         <v>1</v>
       </c>
-      <c r="F8" s="6" t="b">
+      <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8" s="5" t="s">
@@ -1857,8 +1859,8 @@
       <c r="L8" t="b">
         <v>1</v>
       </c>
-      <c r="O8" s="14"/>
-      <c r="P8" s="12"/>
+      <c r="O8" s="18"/>
+      <c r="P8" s="11"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -1897,8 +1899,8 @@
       <c r="L9" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="O9" s="15"/>
-      <c r="P9" s="12" t="s">
+      <c r="O9" s="13"/>
+      <c r="P9" s="11" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1918,29 +1920,29 @@
       <c r="E10" t="b">
         <v>1</v>
       </c>
-      <c r="F10" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G10" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" s="7" t="s">
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I10" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J10" s="7" t="s">
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="K10" s="6" t="b">
+      <c r="K10" t="b">
         <v>1</v>
       </c>
       <c r="L10" t="b">
         <v>1</v>
       </c>
-      <c r="O10" s="15"/>
-      <c r="P10" s="12"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="11"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -1958,7 +1960,7 @@
       <c r="E11" t="b">
         <v>1</v>
       </c>
-      <c r="F11" s="6" t="b">
+      <c r="F11" t="b">
         <v>1</v>
       </c>
       <c r="G11" s="4" t="s">
@@ -1967,20 +1969,20 @@
       <c r="H11" t="b">
         <v>1</v>
       </c>
-      <c r="I11" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J11" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="K11" s="6" t="b">
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" t="b">
         <v>1</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="O11" s="16"/>
-      <c r="P11" s="12" t="s">
+      <c r="O11" s="14"/>
+      <c r="P11" s="11" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2000,29 +2002,29 @@
       <c r="E12" t="b">
         <v>1</v>
       </c>
-      <c r="F12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="K12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="O12" s="16"/>
-      <c r="P12" s="12"/>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" s="14"/>
+      <c r="P12" s="11"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -2040,43 +2042,43 @@
       <c r="E13" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F13" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I13" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J13" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="K13" s="6" t="b">
+      <c r="F13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" t="b">
         <v>1</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="O13" s="17"/>
-      <c r="P13" s="12" t="s">
+      <c r="O13" s="15"/>
+      <c r="P13" s="11" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="A14" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="7" t="s">
         <v>41</v>
       </c>
       <c r="C14" t="s">
         <v>37</v>
       </c>
-      <c r="D14" s="8" t="b">
+      <c r="D14" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E14" s="2" t="s">
@@ -2103,8 +2105,8 @@
       <c r="L14" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="O14" s="17"/>
-      <c r="P14" s="12"/>
+      <c r="O14" s="15"/>
+      <c r="P14" s="11"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -2125,26 +2127,26 @@
       <c r="F15" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G15" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H15" s="7" t="s">
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" s="6" t="s">
         <v>62</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J15" s="7" t="s">
+      <c r="J15" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="K15" s="6" t="b">
+      <c r="K15" t="b">
         <v>1</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="O15" s="18"/>
-      <c r="P15" s="12" t="s">
+      <c r="O15" s="10"/>
+      <c r="P15" s="11" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2164,29 +2166,29 @@
       <c r="E16" t="b">
         <v>1</v>
       </c>
-      <c r="F16" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G16" s="6" t="b">
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" t="b">
         <v>1</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="I16" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J16" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="K16" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L16" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="O16" s="18"/>
-      <c r="P16" s="12"/>
+      <c r="I16" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="O16" s="10"/>
+      <c r="P16" s="11"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -2204,7 +2206,7 @@
       <c r="E17" t="b">
         <v>1</v>
       </c>
-      <c r="F17" s="6" t="b">
+      <c r="F17" t="b">
         <v>1</v>
       </c>
       <c r="G17" s="4" t="s">
@@ -2213,10 +2215,10 @@
       <c r="H17" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="I17" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J17" s="6" t="b">
+      <c r="I17" t="b">
+        <v>1</v>
+      </c>
+      <c r="J17" t="b">
         <v>1</v>
       </c>
       <c r="K17" s="4" t="s">
@@ -2245,7 +2247,7 @@
       <c r="F18" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G18" s="6" t="b">
+      <c r="G18" t="b">
         <v>1</v>
       </c>
       <c r="H18" t="b">
@@ -2254,7 +2256,7 @@
       <c r="I18" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="J18" s="6" t="b">
+      <c r="J18" t="b">
         <v>1</v>
       </c>
       <c r="K18" s="4" t="s">
@@ -2283,22 +2285,22 @@
       <c r="F19" t="b">
         <v>1</v>
       </c>
-      <c r="G19" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H19" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I19" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J19" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="K19" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L19" s="6" t="b">
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" t="b">
+        <v>1</v>
+      </c>
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2321,22 +2323,22 @@
       <c r="F20" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G20" s="6" t="b">
+      <c r="G20" t="b">
         <v>1</v>
       </c>
       <c r="H20" t="b">
         <v>1</v>
       </c>
-      <c r="I20" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J20" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="K20" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L20" s="6" t="b">
+      <c r="I20" t="b">
+        <v>1</v>
+      </c>
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2359,13 +2361,13 @@
       <c r="F21" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G21" s="6" t="b">
+      <c r="G21" t="b">
         <v>1</v>
       </c>
       <c r="H21" t="b">
         <v>1</v>
       </c>
-      <c r="I21" s="6" t="b">
+      <c r="I21" t="b">
         <v>1</v>
       </c>
       <c r="J21" s="2" t="s">
@@ -2374,41 +2376,46 @@
       <c r="K21" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="L21" s="6" t="b">
+      <c r="L21" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D22" s="19" t="s">
+      <c r="B22" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C22" s="12"/>
+      <c r="D22" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="E22" s="19" t="s">
+      <c r="E22" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="F22" s="19" t="s">
+      <c r="F22" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="H22" s="19" t="s">
+      <c r="H22" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="I22" s="19" t="s">
+      <c r="I22" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="J22" s="19" t="s">
+      <c r="J22" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="K22" s="19" t="s">
+      <c r="K22" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="L22" s="19" t="s">
+      <c r="L22" s="9" t="s">
         <v>80</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
+    <mergeCell ref="B22:C22"/>
     <mergeCell ref="O15:O16"/>
     <mergeCell ref="P15:P16"/>
     <mergeCell ref="O2:P2"/>

</xml_diff>